<commit_message>
feat(PDG-61): normalize remaining watchlist date fields via post-norm rules
Add rule rows so every watchlist date field is normalized: DATE_COMPONENT_NORMALIZE for Occupations[] Since/To parts and VesselDetails[].YearBuilt, and defensive DATE_NORMALIZATION (leaves) for Relationships[].StartDate/EndDate and AircraftDetails[].ManufactureDate. No-ops on current data; ready for when those fields are populated.
</commit_message>
<xml_diff>
--- a/data/rules/postNormalization.xlsx
+++ b/data/rules/postNormalization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9032F7F6-0DD9-453C-8708-E0E51E1233A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DAEA36F-894C-4E92-903A-139A2B26C7AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="67">
   <si>
     <t>rule_type</t>
   </si>
@@ -194,6 +194,33 @@
   </si>
   <si>
     <t>leaves=IssuedDate,ExpiryDate</t>
+  </si>
+  <si>
+    <t>DATE_COMPONENT_NORMALIZE</t>
+  </si>
+  <si>
+    <t>Occupations[]</t>
+  </si>
+  <si>
+    <t>day=SinceDay,ToDay|month=SinceMonth,ToMonth|year=SinceYear,ToYear</t>
+  </si>
+  <si>
+    <t>VesselDetails[]</t>
+  </si>
+  <si>
+    <t>year=YearBuilt</t>
+  </si>
+  <si>
+    <t>Relationships[].StartDate</t>
+  </si>
+  <si>
+    <t>leaves=StartDate,EndDate</t>
+  </si>
+  <si>
+    <t>AircraftDetails[].ManufactureDate</t>
+  </si>
+  <si>
+    <t>leaves=ManufactureDate</t>
   </si>
 </sst>
 </file>
@@ -641,15 +668,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F1010"/>
+  <dimension ref="A1:F1014"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.58203125" customWidth="1"/>
     <col min="2" max="2" width="43.83203125" customWidth="1"/>
     <col min="3" max="3" width="19.58203125" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
     <col min="5" max="5" width="19.9140625" customWidth="1"/>
-    <col min="6" max="6" width="33.5" customWidth="1"/>
+    <col min="6" max="6" width="40.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="16" customHeight="1" thickBot="1">
@@ -849,109 +876,97 @@
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:6" s="3" customFormat="1" ht="16" customHeight="1" thickBot="1">
-      <c r="A14" s="9" t="s">
+    <row r="14" spans="1:6" s="3" customFormat="1" ht="33" customHeight="1" thickBot="1">
+      <c r="A14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" s="3" customFormat="1" ht="33" customHeight="1" thickBot="1">
+      <c r="A15" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" s="3" customFormat="1" ht="33" customHeight="1" thickBot="1">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" s="3" customFormat="1" ht="33" customHeight="1" thickBot="1">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="3" customFormat="1" ht="16" customHeight="1" thickBot="1">
+      <c r="A18" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B18" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10" t="s">
+      <c r="C18" s="10"/>
+      <c r="D18" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="E14" s="10"/>
-      <c r="F14" s="9"/>
-    </row>
-    <row r="15" spans="1:6" s="3" customFormat="1" ht="55" customHeight="1" thickBot="1">
-      <c r="A15" s="7" t="s">
+      <c r="E18" s="10"/>
+      <c r="F18" s="9"/>
+    </row>
+    <row r="19" spans="1:6" s="3" customFormat="1" ht="55" customHeight="1" thickBot="1">
+      <c r="A19" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B19" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-    </row>
-    <row r="16" spans="1:6" ht="16" customHeight="1" thickBot="1">
-      <c r="A16" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16" s="5"/>
-      <c r="D16" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F16" s="5"/>
-    </row>
-    <row r="17" spans="1:6" ht="16" customHeight="1" thickBot="1">
-      <c r="A17" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C17" s="5"/>
-      <c r="D17" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F17" s="5"/>
-    </row>
-    <row r="18" spans="1:6" ht="16" customHeight="1" thickBot="1">
-      <c r="A18" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C18" s="5"/>
-      <c r="D18" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="F18" s="5"/>
-    </row>
-    <row r="19" spans="1:6" ht="16" customHeight="1" thickBot="1">
-      <c r="A19" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C19" s="5"/>
-      <c r="D19" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F19" s="5"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:6" ht="16" customHeight="1" thickBot="1">
       <c r="A20" s="4" t="s">
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="4" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F20" s="5"/>
     </row>
@@ -960,14 +975,14 @@
         <v>19</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="4" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F21" s="5"/>
     </row>
@@ -976,14 +991,14 @@
         <v>19</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="4" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="F22" s="5"/>
     </row>
@@ -992,16 +1007,14 @@
         <v>19</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>31</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="C23" s="5"/>
       <c r="D23" s="4" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="F23" s="5"/>
     </row>
@@ -1010,16 +1023,14 @@
         <v>19</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>31</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="C24" s="5"/>
       <c r="D24" s="4" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="F24" s="5"/>
     </row>
@@ -1028,53 +1039,89 @@
         <v>19</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="4" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="F25" s="5"/>
     </row>
     <row r="26" spans="1:6" ht="16" customHeight="1" thickBot="1">
       <c r="A26" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" s="5"/>
+      <c r="D26" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F26" s="5"/>
+    </row>
+    <row r="27" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A27" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F27" s="5"/>
+    </row>
+    <row r="28" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A28" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F28" s="5"/>
+    </row>
+    <row r="29" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A29" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C29" s="5"/>
+      <c r="D29" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F29" s="5"/>
+    </row>
+    <row r="30" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A30" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-    </row>
-    <row r="27" spans="1:6" ht="16" customHeight="1" thickBot="1">
-      <c r="A27" s="5"/>
-      <c r="B27" s="5"/>
-      <c r="C27" s="5"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-    </row>
-    <row r="28" spans="1:6" ht="16" customHeight="1" thickBot="1">
-      <c r="A28" s="5"/>
-      <c r="B28" s="5"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
-    </row>
-    <row r="29" spans="1:6" ht="16" customHeight="1" thickBot="1">
-      <c r="A29" s="5"/>
-      <c r="B29" s="5"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
-    </row>
-    <row r="30" spans="1:6" ht="16" customHeight="1" thickBot="1">
-      <c r="A30" s="5"/>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
@@ -8897,9 +8944,41 @@
       <c r="E1007" s="5"/>
       <c r="F1007" s="5"/>
     </row>
-    <row r="1008" spans="1:6" ht="16" customHeight="1"/>
-    <row r="1009" ht="16" customHeight="1"/>
-    <row r="1010" ht="16" customHeight="1"/>
+    <row r="1008" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A1008" s="5"/>
+      <c r="B1008" s="5"/>
+      <c r="C1008" s="5"/>
+      <c r="D1008" s="5"/>
+      <c r="E1008" s="5"/>
+      <c r="F1008" s="5"/>
+    </row>
+    <row r="1009" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A1009" s="5"/>
+      <c r="B1009" s="5"/>
+      <c r="C1009" s="5"/>
+      <c r="D1009" s="5"/>
+      <c r="E1009" s="5"/>
+      <c r="F1009" s="5"/>
+    </row>
+    <row r="1010" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A1010" s="5"/>
+      <c r="B1010" s="5"/>
+      <c r="C1010" s="5"/>
+      <c r="D1010" s="5"/>
+      <c r="E1010" s="5"/>
+      <c r="F1010" s="5"/>
+    </row>
+    <row r="1011" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A1011" s="5"/>
+      <c r="B1011" s="5"/>
+      <c r="C1011" s="5"/>
+      <c r="D1011" s="5"/>
+      <c r="E1011" s="5"/>
+      <c r="F1011" s="5"/>
+    </row>
+    <row r="1012" spans="1:6" ht="16" customHeight="1"/>
+    <row r="1013" spans="1:6" ht="16" customHeight="1"/>
+    <row r="1014" spans="1:6" ht="16" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat(PDG-73): add AFDB-DEBARRED-ENTITIES watchlist source
Download the AfDB debarred-entities JSON feed through the Cloudflare bypass, split aliases out of the name, derive status from the From/To dates instead of the unreliable ONGOING note, and decode HTML entities in names, aliases and country names.
</commit_message>
<xml_diff>
--- a/data/rules/postNormalization.xlsx
+++ b/data/rules/postNormalization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DAEA36F-894C-4E92-903A-139A2B26C7AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA438332-F660-4AE0-8E61-6D8195AE41E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="67">
   <si>
     <t>rule_type</t>
   </si>
@@ -324,7 +324,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -353,6 +353,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -668,7 +671,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F1014"/>
+  <dimension ref="A1:F1017"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="28.58203125" customWidth="1"/>
@@ -954,64 +957,52 @@
       <c r="E19" s="8"/>
       <c r="F19" s="8"/>
     </row>
-    <row r="20" spans="1:6" ht="16" customHeight="1" thickBot="1">
-      <c r="A20" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20" s="4" t="s">
+    <row r="20" spans="1:6" s="3" customFormat="1" ht="28" customHeight="1" thickBot="1">
+      <c r="A20" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="5"/>
-      <c r="D20" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F20" s="5"/>
-    </row>
-    <row r="21" spans="1:6" ht="16" customHeight="1" thickBot="1">
-      <c r="A21" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C21" s="5"/>
-      <c r="D21" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F21" s="5"/>
-    </row>
-    <row r="22" spans="1:6" ht="16" customHeight="1" thickBot="1">
-      <c r="A22" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C22" s="5"/>
-      <c r="D22" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="F22" s="5"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+    </row>
+    <row r="21" spans="1:6" s="3" customFormat="1" ht="35.5" customHeight="1" thickBot="1">
+      <c r="A21" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" s="11"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+    </row>
+    <row r="22" spans="1:6" s="3" customFormat="1" ht="17" customHeight="1" thickBot="1">
+      <c r="A22" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" s="11"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
     </row>
     <row r="23" spans="1:6" ht="16" customHeight="1" thickBot="1">
       <c r="A23" s="4" t="s">
         <v>19</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="4" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>22</v>
@@ -1023,11 +1014,11 @@
         <v>19</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="4" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>24</v>
@@ -1039,11 +1030,11 @@
         <v>19</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="4" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>26</v>
@@ -1055,14 +1046,14 @@
         <v>19</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="4" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="F26" s="5"/>
     </row>
@@ -1071,16 +1062,14 @@
         <v>19</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>31</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="C27" s="5"/>
       <c r="D27" s="4" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="F27" s="5"/>
     </row>
@@ -1089,16 +1078,14 @@
         <v>19</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>31</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="C28" s="5"/>
       <c r="D28" s="4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="F28" s="5"/>
     </row>
@@ -1107,45 +1094,73 @@
         <v>19</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F29" s="5"/>
     </row>
     <row r="30" spans="1:6" ht="16" customHeight="1" thickBot="1">
       <c r="A30" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F30" s="5"/>
+    </row>
+    <row r="31" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A31" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F31" s="5"/>
+    </row>
+    <row r="32" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A32" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C32" s="5"/>
+      <c r="D32" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F32" s="5"/>
+    </row>
+    <row r="33" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A33" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B30" s="5"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
-    </row>
-    <row r="31" spans="1:6" ht="16" customHeight="1" thickBot="1">
-      <c r="A31" s="5"/>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
-    </row>
-    <row r="32" spans="1:6" ht="16" customHeight="1" thickBot="1">
-      <c r="A32" s="5"/>
-      <c r="B32" s="5"/>
-      <c r="C32" s="5"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
-    </row>
-    <row r="33" spans="1:6" ht="16" customHeight="1" thickBot="1">
-      <c r="A33" s="5"/>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
       <c r="D33" s="5"/>
@@ -8976,9 +8991,33 @@
       <c r="E1011" s="5"/>
       <c r="F1011" s="5"/>
     </row>
-    <row r="1012" spans="1:6" ht="16" customHeight="1"/>
-    <row r="1013" spans="1:6" ht="16" customHeight="1"/>
-    <row r="1014" spans="1:6" ht="16" customHeight="1"/>
+    <row r="1012" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A1012" s="5"/>
+      <c r="B1012" s="5"/>
+      <c r="C1012" s="5"/>
+      <c r="D1012" s="5"/>
+      <c r="E1012" s="5"/>
+      <c r="F1012" s="5"/>
+    </row>
+    <row r="1013" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A1013" s="5"/>
+      <c r="B1013" s="5"/>
+      <c r="C1013" s="5"/>
+      <c r="D1013" s="5"/>
+      <c r="E1013" s="5"/>
+      <c r="F1013" s="5"/>
+    </row>
+    <row r="1014" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A1014" s="5"/>
+      <c r="B1014" s="5"/>
+      <c r="C1014" s="5"/>
+      <c r="D1014" s="5"/>
+      <c r="E1014" s="5"/>
+      <c r="F1014" s="5"/>
+    </row>
+    <row r="1015" spans="1:6" ht="16" customHeight="1"/>
+    <row r="1016" spans="1:6" ht="16" customHeight="1"/>
+    <row r="1017" spans="1:6" ht="16" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
fix(normalization): suppress empty notes and resolve country names
</commit_message>
<xml_diff>
--- a/data/rules/postNormalization.xlsx
+++ b/data/rules/postNormalization.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA438332-F660-4AE0-8E61-6D8195AE41E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61AFC66B-A2C7-4FDA-B328-737E9CCB728A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="68">
   <si>
     <t>rule_type</t>
   </si>
@@ -221,6 +221,9 @@
   </si>
   <si>
     <t>leaves=ManufactureDate</t>
+  </si>
+  <si>
+    <t>COUNTRY_NAME</t>
   </si>
 </sst>
 </file>
@@ -671,14 +674,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F1017"/>
+  <dimension ref="A1:F1018"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="28.58203125" customWidth="1"/>
     <col min="2" max="2" width="43.83203125" customWidth="1"/>
     <col min="3" max="3" width="19.58203125" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="5" width="19.9140625" customWidth="1"/>
+    <col min="5" max="5" width="21.25" customWidth="1"/>
     <col min="6" max="6" width="40.5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1146,29 +1149,39 @@
         <v>19</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C32" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>31</v>
+      </c>
       <c r="D32" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="F32" s="5"/>
     </row>
     <row r="33" spans="1:6" ht="16" customHeight="1" thickBot="1">
       <c r="A33" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C33" s="5"/>
+      <c r="D33" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F33" s="5"/>
+    </row>
+    <row r="34" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A34" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B33" s="5"/>
-      <c r="C33" s="5"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-    </row>
-    <row r="34" spans="1:6" ht="16" customHeight="1" thickBot="1">
-      <c r="A34" s="5"/>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
       <c r="D34" s="5"/>
@@ -9015,9 +9028,17 @@
       <c r="E1014" s="5"/>
       <c r="F1014" s="5"/>
     </row>
-    <row r="1015" spans="1:6" ht="16" customHeight="1"/>
+    <row r="1015" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A1015" s="5"/>
+      <c r="B1015" s="5"/>
+      <c r="C1015" s="5"/>
+      <c r="D1015" s="5"/>
+      <c r="E1015" s="5"/>
+      <c r="F1015" s="5"/>
+    </row>
     <row r="1016" spans="1:6" ht="16" customHeight="1"/>
     <row r="1017" spans="1:6" ht="16" customHeight="1"/>
+    <row r="1018" spans="1:6" ht="16" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
fix(normalization): sanitize invisible characters and occupation notes
</commit_message>
<xml_diff>
--- a/data/rules/postNormalization.xlsx
+++ b/data/rules/postNormalization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61AFC66B-A2C7-4FDA-B328-737E9CCB728A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{912E9372-5BA3-43ED-B5FD-E1B118162B24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="69">
   <si>
     <t>rule_type</t>
   </si>
@@ -224,6 +224,9 @@
   </si>
   <si>
     <t>COUNTRY_NAME</t>
+  </si>
+  <si>
+    <t>Occupations[].Note</t>
   </si>
 </sst>
 </file>
@@ -674,7 +677,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F1018"/>
+  <dimension ref="A1:F1019"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="28.58203125" customWidth="1"/>
@@ -1180,16 +1183,20 @@
     </row>
     <row r="34" spans="1:6" ht="16" customHeight="1" thickBot="1">
       <c r="A34" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C34" s="5"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="5"/>
+    </row>
+    <row r="35" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A35" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B34" s="5"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5"/>
-    </row>
-    <row r="35" spans="1:6" ht="16" customHeight="1" thickBot="1">
-      <c r="A35" s="5"/>
       <c r="B35" s="5"/>
       <c r="C35" s="5"/>
       <c r="D35" s="5"/>
@@ -9036,9 +9043,17 @@
       <c r="E1015" s="5"/>
       <c r="F1015" s="5"/>
     </row>
-    <row r="1016" spans="1:6" ht="16" customHeight="1"/>
+    <row r="1016" spans="1:6" ht="16" customHeight="1" thickBot="1">
+      <c r="A1016" s="5"/>
+      <c r="B1016" s="5"/>
+      <c r="C1016" s="5"/>
+      <c r="D1016" s="5"/>
+      <c r="E1016" s="5"/>
+      <c r="F1016" s="5"/>
+    </row>
     <row r="1017" spans="1:6" ht="16" customHeight="1"/>
     <row r="1018" spans="1:6" ht="16" customHeight="1"/>
+    <row r="1019" spans="1:6" ht="16" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>